<commit_message>
Link dei template Excel di nuovo funzionanti, e template con la colonna "Gruppo"
1. proxy.ts: il matcher esclude anche i file .xlsx. Prima una richiesta a
   /template-transazioni.xlsx passava per next-intl, veniva reindirizzata a
   /it/template-transazioni.xlsx, che non esiste, e il link "Scarica
   template vuoto" non scaricava nulla. Ora tutti e quattro i template
   rispondono 200.
2. Template italiani aggiornati a mano: la colonna si chiama "Gruppo", e la
   nota del template liquidità dice "nome di un gruppo esistente".
3. scripts/genera-template-excel.mjs: la nota inglese dice "name of an
   existing group". Template inglesi rigenerati: intestazione e nota dicono
   "Group", e l'import legge tutti e quattro i template senza intestazioni
   sconosciute.
</commit_message>
<xml_diff>
--- a/public/template-transazioni-liquidita-en.xlsx
+++ b/public/template-transazioni-liquidita-en.xlsx
@@ -424,7 +424,7 @@
         <v>Withheld tax</v>
       </c>
       <c r="F1" t="str">
-        <v>Container</v>
+        <v>Group</v>
       </c>
     </row>
     <row r="2">
@@ -479,7 +479,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>- Container: name of an existing container, or leave empty.</v>
+        <v>- Group: name of an existing group, or leave empty.</v>
       </c>
     </row>
     <row r="11">

</xml_diff>